<commit_message>
Capture all 277 TRGs from the homepage
Parser dropped http:// links, sub-page links, external sites and entries without
links (278 numbered entries, 277 distinct). Adds packaging script and notes for
TRGs without their own page.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VuHePFv7oto5SNMHb2pbjZ
</commit_message>
<xml_diff>
--- a/forms/trg/Formulir_TRG_asds.xlsx
+++ b/forms/trg/Formulir_TRG_asds.xlsx
@@ -564,7 +564,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Formulir kelengkapan data: Applied Statistics and Data Science  Research Group</t>
+          <t>Formulir kelengkapan data: Applied Statistics and Data Science Research Group</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Anggota Applied Statistics and Data Science  Research Group</t>
+          <t>Anggota Applied Statistics and Data Science Research Group</t>
         </is>
       </c>
     </row>
@@ -1953,7 +1953,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Profil Applied Statistics and Data Science  Research Group</t>
+          <t>Profil Applied Statistics and Data Science Research Group</t>
         </is>
       </c>
     </row>

</xml_diff>